<commit_message>
add inventory item properties, log filtering, and seed script fix
Add reorder_status, on_hand_qty, in_transit_qty, and min_order_qty
properties to InventoryItem. Add DjangoFilterBackend to InventoryLogViewSet
with received_date__isnull filter. Fix column mapping in seed_inventory_logs
command. Add UpdateModelMixin to InventoryLogViewSet.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/jinx-1.xlsx
+++ b/files/jinx-1.xlsx
@@ -9,11 +9,12 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Current Inventory'!$A$3:$M$57</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Inventory Log'!$A$3:$H$1028</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="ohTFeTf6YzYjs8crz0NCApfek7348oNMRXVkVmrKR6o="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="mUQeYl6i4zBcjDYhHSJfiy2oNQuwI/GyHtndIhbkWh8="/>
     </ext>
   </extLst>
 </workbook>
@@ -7962,7 +7963,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="1">
       <c r="A4" s="46">
         <v>46097.0</v>
       </c>
@@ -8006,7 +8007,7 @@
       <c r="Z4" s="48"/>
       <c r="AA4" s="48"/>
     </row>
-    <row r="5">
+    <row r="5" hidden="1">
       <c r="A5" s="46">
         <v>46097.0</v>
       </c>
@@ -8050,7 +8051,7 @@
       <c r="Z5" s="48"/>
       <c r="AA5" s="48"/>
     </row>
-    <row r="6">
+    <row r="6" hidden="1">
       <c r="A6" s="46">
         <v>46097.0</v>
       </c>
@@ -8094,7 +8095,7 @@
       <c r="Z6" s="48"/>
       <c r="AA6" s="48"/>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" s="46">
         <v>46097.0</v>
       </c>
@@ -8138,7 +8139,7 @@
       <c r="Z7" s="48"/>
       <c r="AA7" s="48"/>
     </row>
-    <row r="8">
+    <row r="8" hidden="1">
       <c r="A8" s="46">
         <v>46097.0</v>
       </c>
@@ -8182,7 +8183,7 @@
       <c r="Z8" s="48"/>
       <c r="AA8" s="48"/>
     </row>
-    <row r="9">
+    <row r="9" hidden="1">
       <c r="A9" s="46">
         <v>46097.0</v>
       </c>
@@ -8226,7 +8227,7 @@
       <c r="Z9" s="48"/>
       <c r="AA9" s="48"/>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" s="46">
         <v>46097.0</v>
       </c>
@@ -8270,7 +8271,7 @@
       <c r="Z10" s="48"/>
       <c r="AA10" s="48"/>
     </row>
-    <row r="11">
+    <row r="11" hidden="1">
       <c r="A11" s="46">
         <v>46097.0</v>
       </c>
@@ -8314,7 +8315,7 @@
       <c r="Z11" s="48"/>
       <c r="AA11" s="48"/>
     </row>
-    <row r="12">
+    <row r="12" hidden="1">
       <c r="A12" s="46">
         <v>46097.0</v>
       </c>
@@ -8358,7 +8359,7 @@
       <c r="Z12" s="48"/>
       <c r="AA12" s="48"/>
     </row>
-    <row r="13">
+    <row r="13" hidden="1">
       <c r="A13" s="46">
         <v>46097.0</v>
       </c>
@@ -8402,7 +8403,7 @@
       <c r="Z13" s="48"/>
       <c r="AA13" s="48"/>
     </row>
-    <row r="14">
+    <row r="14" hidden="1">
       <c r="A14" s="46">
         <v>46097.0</v>
       </c>
@@ -8446,7 +8447,7 @@
       <c r="Z14" s="48"/>
       <c r="AA14" s="48"/>
     </row>
-    <row r="15">
+    <row r="15" hidden="1">
       <c r="A15" s="46">
         <v>46097.0</v>
       </c>
@@ -8490,7 +8491,7 @@
       <c r="Z15" s="48"/>
       <c r="AA15" s="48"/>
     </row>
-    <row r="16">
+    <row r="16" hidden="1">
       <c r="A16" s="46">
         <v>46097.0</v>
       </c>
@@ -8534,7 +8535,7 @@
       <c r="Z16" s="48"/>
       <c r="AA16" s="48"/>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" s="46">
         <v>46097.0</v>
       </c>
@@ -8578,7 +8579,7 @@
       <c r="Z17" s="48"/>
       <c r="AA17" s="48"/>
     </row>
-    <row r="18">
+    <row r="18" hidden="1">
       <c r="A18" s="46">
         <v>46097.0</v>
       </c>
@@ -8622,7 +8623,7 @@
       <c r="Z18" s="48"/>
       <c r="AA18" s="48"/>
     </row>
-    <row r="19">
+    <row r="19" hidden="1">
       <c r="A19" s="46">
         <v>46097.0</v>
       </c>
@@ -8666,7 +8667,7 @@
       <c r="Z19" s="48"/>
       <c r="AA19" s="48"/>
     </row>
-    <row r="20">
+    <row r="20" hidden="1">
       <c r="A20" s="46">
         <v>46097.0</v>
       </c>
@@ -8710,7 +8711,7 @@
       <c r="Z20" s="48"/>
       <c r="AA20" s="48"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" hidden="1" customHeight="1">
       <c r="A21" s="46">
         <v>46097.0</v>
       </c>
@@ -8754,7 +8755,7 @@
       <c r="Z21" s="48"/>
       <c r="AA21" s="48"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" hidden="1" customHeight="1">
       <c r="A22" s="46">
         <v>46097.0</v>
       </c>
@@ -8798,7 +8799,7 @@
       <c r="Z22" s="48"/>
       <c r="AA22" s="48"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" hidden="1" customHeight="1">
       <c r="A23" s="46">
         <v>46097.0</v>
       </c>
@@ -8842,7 +8843,7 @@
       <c r="Z23" s="48"/>
       <c r="AA23" s="48"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" hidden="1" customHeight="1">
       <c r="A24" s="46">
         <v>46097.0</v>
       </c>
@@ -8886,7 +8887,7 @@
       <c r="Z24" s="48"/>
       <c r="AA24" s="48"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="15.75" hidden="1" customHeight="1">
       <c r="A25" s="46">
         <v>46097.0</v>
       </c>
@@ -8930,7 +8931,7 @@
       <c r="Z25" s="48"/>
       <c r="AA25" s="48"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="15.75" hidden="1" customHeight="1">
       <c r="A26" s="46">
         <v>46097.0</v>
       </c>
@@ -8974,7 +8975,7 @@
       <c r="Z26" s="48"/>
       <c r="AA26" s="48"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="15.75" hidden="1" customHeight="1">
       <c r="A27" s="46">
         <v>46097.0</v>
       </c>
@@ -9018,7 +9019,7 @@
       <c r="Z27" s="48"/>
       <c r="AA27" s="48"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="15.75" hidden="1" customHeight="1">
       <c r="A28" s="46">
         <v>46097.0</v>
       </c>
@@ -9062,7 +9063,7 @@
       <c r="Z28" s="48"/>
       <c r="AA28" s="48"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" hidden="1" customHeight="1">
       <c r="A29" s="46">
         <v>46097.0</v>
       </c>
@@ -9106,7 +9107,7 @@
       <c r="Z29" s="48"/>
       <c r="AA29" s="48"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="15.75" hidden="1" customHeight="1">
       <c r="A30" s="46">
         <v>46097.0</v>
       </c>
@@ -9150,7 +9151,7 @@
       <c r="Z30" s="48"/>
       <c r="AA30" s="48"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" hidden="1" customHeight="1">
       <c r="A31" s="46">
         <v>46097.0</v>
       </c>
@@ -9194,7 +9195,7 @@
       <c r="Z31" s="48"/>
       <c r="AA31" s="48"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" hidden="1" customHeight="1">
       <c r="A32" s="46">
         <v>46097.0</v>
       </c>
@@ -9238,7 +9239,7 @@
       <c r="Z32" s="48"/>
       <c r="AA32" s="48"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" hidden="1" customHeight="1">
       <c r="A33" s="46">
         <v>46097.0</v>
       </c>
@@ -9282,7 +9283,7 @@
       <c r="Z33" s="48"/>
       <c r="AA33" s="48"/>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="15.75" hidden="1" customHeight="1">
       <c r="A34" s="46">
         <v>46097.0</v>
       </c>
@@ -9326,7 +9327,7 @@
       <c r="Z34" s="48"/>
       <c r="AA34" s="48"/>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="15.75" hidden="1" customHeight="1">
       <c r="A35" s="46">
         <v>46097.0</v>
       </c>
@@ -9370,7 +9371,7 @@
       <c r="Z35" s="48"/>
       <c r="AA35" s="48"/>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="15.75" hidden="1" customHeight="1">
       <c r="A36" s="46">
         <v>46097.0</v>
       </c>
@@ -9414,7 +9415,7 @@
       <c r="Z36" s="48"/>
       <c r="AA36" s="48"/>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" hidden="1" customHeight="1">
       <c r="A37" s="46">
         <v>46097.0</v>
       </c>
@@ -9458,7 +9459,7 @@
       <c r="Z37" s="48"/>
       <c r="AA37" s="48"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" hidden="1" customHeight="1">
       <c r="A38" s="46">
         <v>46097.0</v>
       </c>
@@ -9502,7 +9503,7 @@
       <c r="Z38" s="48"/>
       <c r="AA38" s="48"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" hidden="1" customHeight="1">
       <c r="A39" s="46">
         <v>46097.0</v>
       </c>
@@ -9546,7 +9547,7 @@
       <c r="Z39" s="48"/>
       <c r="AA39" s="48"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" hidden="1" customHeight="1">
       <c r="A40" s="46">
         <v>46097.0</v>
       </c>
@@ -9590,7 +9591,7 @@
       <c r="Z40" s="48"/>
       <c r="AA40" s="48"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" hidden="1" customHeight="1">
       <c r="A41" s="46">
         <v>46097.0</v>
       </c>
@@ -9634,7 +9635,7 @@
       <c r="Z41" s="48"/>
       <c r="AA41" s="48"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="15.75" hidden="1" customHeight="1">
       <c r="A42" s="46">
         <v>46097.0</v>
       </c>
@@ -9678,7 +9679,7 @@
       <c r="Z42" s="48"/>
       <c r="AA42" s="48"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="15.75" hidden="1" customHeight="1">
       <c r="A43" s="46">
         <v>46097.0</v>
       </c>
@@ -9722,7 +9723,7 @@
       <c r="Z43" s="48"/>
       <c r="AA43" s="48"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" hidden="1" customHeight="1">
       <c r="A44" s="46">
         <v>46097.0</v>
       </c>
@@ -9766,7 +9767,7 @@
       <c r="Z44" s="48"/>
       <c r="AA44" s="48"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" hidden="1" customHeight="1">
       <c r="A45" s="46">
         <v>46097.0</v>
       </c>
@@ -9810,7 +9811,7 @@
       <c r="Z45" s="48"/>
       <c r="AA45" s="48"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="15.75" hidden="1" customHeight="1">
       <c r="A46" s="46">
         <v>46097.0</v>
       </c>
@@ -9854,7 +9855,7 @@
       <c r="Z46" s="48"/>
       <c r="AA46" s="48"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="15.75" hidden="1" customHeight="1">
       <c r="A47" s="46">
         <v>46097.0</v>
       </c>
@@ -9898,7 +9899,7 @@
       <c r="Z47" s="48"/>
       <c r="AA47" s="48"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="15.75" hidden="1" customHeight="1">
       <c r="A48" s="46">
         <v>46097.0</v>
       </c>
@@ -9942,7 +9943,7 @@
       <c r="Z48" s="48"/>
       <c r="AA48" s="48"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="15.75" hidden="1" customHeight="1">
       <c r="A49" s="46">
         <v>46097.0</v>
       </c>
@@ -9986,7 +9987,7 @@
       <c r="Z49" s="48"/>
       <c r="AA49" s="48"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="15.75" hidden="1" customHeight="1">
       <c r="A50" s="46">
         <v>46097.0</v>
       </c>
@@ -10028,11 +10029,13 @@
       <c r="Z50" s="48"/>
       <c r="AA50" s="48"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="15.75" hidden="1" customHeight="1">
       <c r="A51" s="46">
         <v>46104.0</v>
       </c>
-      <c r="B51" s="52"/>
+      <c r="B51" s="46">
+        <v>46109.0</v>
+      </c>
       <c r="C51" s="30" t="s">
         <v>61</v>
       </c>
@@ -10068,11 +10071,13 @@
       <c r="Z51" s="48"/>
       <c r="AA51" s="48"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="15.75" hidden="1" customHeight="1">
       <c r="A52" s="46">
         <v>46104.0</v>
       </c>
-      <c r="B52" s="52"/>
+      <c r="B52" s="46">
+        <v>46109.0</v>
+      </c>
       <c r="C52" s="49" t="s">
         <v>103</v>
       </c>
@@ -10108,7 +10113,7 @@
       <c r="Z52" s="48"/>
       <c r="AA52" s="48"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" ht="15.75" hidden="1" customHeight="1">
       <c r="A53" s="46">
         <v>46101.0</v>
       </c>
@@ -10150,7 +10155,7 @@
       <c r="Z53" s="48"/>
       <c r="AA53" s="48"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1">
+    <row r="54" ht="15.75" hidden="1" customHeight="1">
       <c r="A54" s="46">
         <v>46101.0</v>
       </c>
@@ -10192,7 +10197,7 @@
       <c r="Z54" s="48"/>
       <c r="AA54" s="48"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1">
+    <row r="55" ht="15.75" hidden="1" customHeight="1">
       <c r="A55" s="46">
         <v>46101.0</v>
       </c>
@@ -10234,7 +10239,7 @@
       <c r="Z55" s="48"/>
       <c r="AA55" s="48"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1">
+    <row r="56" ht="15.75" hidden="1" customHeight="1">
       <c r="A56" s="46">
         <v>46101.0</v>
       </c>
@@ -10276,7 +10281,7 @@
       <c r="Z56" s="48"/>
       <c r="AA56" s="48"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1">
+    <row r="57" ht="15.75" hidden="1" customHeight="1">
       <c r="A57" s="46">
         <v>46101.0</v>
       </c>
@@ -10318,7 +10323,7 @@
       <c r="Z57" s="48"/>
       <c r="AA57" s="48"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1">
+    <row r="58" ht="15.75" hidden="1" customHeight="1">
       <c r="A58" s="46">
         <v>46101.0</v>
       </c>
@@ -10360,7 +10365,7 @@
       <c r="Z58" s="48"/>
       <c r="AA58" s="48"/>
     </row>
-    <row r="59" ht="15.75" customHeight="1">
+    <row r="59" ht="15.75" hidden="1" customHeight="1">
       <c r="A59" s="46">
         <v>46101.0</v>
       </c>
@@ -10402,7 +10407,7 @@
       <c r="Z59" s="48"/>
       <c r="AA59" s="48"/>
     </row>
-    <row r="60" ht="15.75" customHeight="1">
+    <row r="60" ht="15.75" hidden="1" customHeight="1">
       <c r="A60" s="46">
         <v>46101.0</v>
       </c>
@@ -10444,7 +10449,7 @@
       <c r="Z60" s="48"/>
       <c r="AA60" s="48"/>
     </row>
-    <row r="61" ht="15.75" customHeight="1">
+    <row r="61" ht="15.75" hidden="1" customHeight="1">
       <c r="A61" s="46">
         <v>46102.0</v>
       </c>
@@ -10486,7 +10491,7 @@
       <c r="Z61" s="48"/>
       <c r="AA61" s="48"/>
     </row>
-    <row r="62" ht="15.75" customHeight="1">
+    <row r="62" ht="15.75" hidden="1" customHeight="1">
       <c r="A62" s="46">
         <v>46102.0</v>
       </c>
@@ -10528,7 +10533,7 @@
       <c r="Z62" s="48"/>
       <c r="AA62" s="48"/>
     </row>
-    <row r="63" ht="15.75" customHeight="1">
+    <row r="63" ht="15.75" hidden="1" customHeight="1">
       <c r="A63" s="46">
         <v>46102.0</v>
       </c>
@@ -10570,7 +10575,7 @@
       <c r="Z63" s="48"/>
       <c r="AA63" s="48"/>
     </row>
-    <row r="64" ht="15.75" customHeight="1">
+    <row r="64" ht="15.75" hidden="1" customHeight="1">
       <c r="A64" s="46">
         <v>46102.0</v>
       </c>
@@ -10612,7 +10617,7 @@
       <c r="Z64" s="48"/>
       <c r="AA64" s="48"/>
     </row>
-    <row r="65" ht="15.75" customHeight="1">
+    <row r="65" ht="15.75" hidden="1" customHeight="1">
       <c r="A65" s="46">
         <v>46102.0</v>
       </c>
@@ -10654,7 +10659,7 @@
       <c r="Z65" s="48"/>
       <c r="AA65" s="48"/>
     </row>
-    <row r="66" ht="15.75" customHeight="1">
+    <row r="66" ht="15.75" hidden="1" customHeight="1">
       <c r="A66" s="46">
         <v>46102.0</v>
       </c>
@@ -10696,7 +10701,7 @@
       <c r="Z66" s="48"/>
       <c r="AA66" s="48"/>
     </row>
-    <row r="67" ht="15.75" customHeight="1">
+    <row r="67" ht="15.75" hidden="1" customHeight="1">
       <c r="A67" s="46">
         <v>46102.0</v>
       </c>
@@ -10738,7 +10743,7 @@
       <c r="Z67" s="48"/>
       <c r="AA67" s="48"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1">
+    <row r="68" ht="15.75" hidden="1" customHeight="1">
       <c r="A68" s="46">
         <v>46102.0</v>
       </c>
@@ -10780,7 +10785,7 @@
       <c r="Z68" s="48"/>
       <c r="AA68" s="48"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1">
+    <row r="69" ht="15.75" hidden="1" customHeight="1">
       <c r="A69" s="46">
         <v>46102.0</v>
       </c>
@@ -10822,7 +10827,7 @@
       <c r="Z69" s="48"/>
       <c r="AA69" s="48"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1">
+    <row r="70" ht="15.75" hidden="1" customHeight="1">
       <c r="A70" s="46">
         <v>46102.0</v>
       </c>
@@ -10864,7 +10869,7 @@
       <c r="Z70" s="48"/>
       <c r="AA70" s="48"/>
     </row>
-    <row r="71" ht="15.75" customHeight="1">
+    <row r="71" ht="15.75" hidden="1" customHeight="1">
       <c r="A71" s="46">
         <v>46102.0</v>
       </c>
@@ -10906,7 +10911,7 @@
       <c r="Z71" s="48"/>
       <c r="AA71" s="48"/>
     </row>
-    <row r="72" ht="15.75" customHeight="1">
+    <row r="72" ht="15.75" hidden="1" customHeight="1">
       <c r="A72" s="46">
         <v>46102.0</v>
       </c>
@@ -10948,7 +10953,7 @@
       <c r="Z72" s="48"/>
       <c r="AA72" s="48"/>
     </row>
-    <row r="73" ht="15.75" customHeight="1">
+    <row r="73" ht="15.75" hidden="1" customHeight="1">
       <c r="A73" s="46">
         <v>46102.0</v>
       </c>
@@ -10990,7 +10995,7 @@
       <c r="Z73" s="48"/>
       <c r="AA73" s="48"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1">
+    <row r="74" ht="15.75" hidden="1" customHeight="1">
       <c r="A74" s="46">
         <v>46102.0</v>
       </c>
@@ -11032,7 +11037,7 @@
       <c r="Z74" s="48"/>
       <c r="AA74" s="48"/>
     </row>
-    <row r="75" ht="15.75" customHeight="1">
+    <row r="75" ht="15.75" hidden="1" customHeight="1">
       <c r="A75" s="46">
         <v>46102.0</v>
       </c>
@@ -11074,7 +11079,7 @@
       <c r="Z75" s="48"/>
       <c r="AA75" s="48"/>
     </row>
-    <row r="76" ht="15.75" customHeight="1">
+    <row r="76" ht="15.75" hidden="1" customHeight="1">
       <c r="A76" s="46">
         <v>46102.0</v>
       </c>
@@ -11116,7 +11121,7 @@
       <c r="Z76" s="48"/>
       <c r="AA76" s="48"/>
     </row>
-    <row r="77" ht="15.75" customHeight="1">
+    <row r="77" ht="15.75" hidden="1" customHeight="1">
       <c r="A77" s="46">
         <v>46102.0</v>
       </c>
@@ -11158,7 +11163,7 @@
       <c r="Z77" s="48"/>
       <c r="AA77" s="48"/>
     </row>
-    <row r="78" ht="15.75" customHeight="1">
+    <row r="78" ht="15.75" hidden="1" customHeight="1">
       <c r="A78" s="46">
         <v>46102.0</v>
       </c>
@@ -11200,7 +11205,7 @@
       <c r="Z78" s="48"/>
       <c r="AA78" s="48"/>
     </row>
-    <row r="79" ht="15.75" customHeight="1">
+    <row r="79" ht="15.75" hidden="1" customHeight="1">
       <c r="A79" s="46">
         <v>46102.0</v>
       </c>
@@ -11242,7 +11247,7 @@
       <c r="Z79" s="48"/>
       <c r="AA79" s="48"/>
     </row>
-    <row r="80" ht="15.75" customHeight="1">
+    <row r="80" ht="15.75" hidden="1" customHeight="1">
       <c r="A80" s="46">
         <v>46102.0</v>
       </c>
@@ -11284,7 +11289,7 @@
       <c r="Z80" s="48"/>
       <c r="AA80" s="48"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1">
+    <row r="81" ht="15.75" hidden="1" customHeight="1">
       <c r="A81" s="46">
         <v>46102.0</v>
       </c>
@@ -11326,7 +11331,7 @@
       <c r="Z81" s="48"/>
       <c r="AA81" s="48"/>
     </row>
-    <row r="82" ht="15.75" customHeight="1">
+    <row r="82" ht="15.75" hidden="1" customHeight="1">
       <c r="A82" s="46">
         <v>46102.0</v>
       </c>
@@ -11368,7 +11373,7 @@
       <c r="Z82" s="48"/>
       <c r="AA82" s="48"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1">
+    <row r="83" ht="15.75" hidden="1" customHeight="1">
       <c r="A83" s="46">
         <v>46102.0</v>
       </c>
@@ -11450,7 +11455,7 @@
       <c r="Z84" s="48"/>
       <c r="AA84" s="48"/>
     </row>
-    <row r="85" ht="15.75" customHeight="1">
+    <row r="85" ht="15.75" hidden="1" customHeight="1">
       <c r="A85" s="46">
         <v>46104.0</v>
       </c>
@@ -11492,7 +11497,7 @@
       <c r="Z85" s="48"/>
       <c r="AA85" s="48"/>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
+    <row r="86" ht="15.75" hidden="1" customHeight="1">
       <c r="A86" s="46">
         <v>46104.0</v>
       </c>
@@ -11534,7 +11539,7 @@
       <c r="Z86" s="48"/>
       <c r="AA86" s="48"/>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
+    <row r="87" ht="15.75" hidden="1" customHeight="1">
       <c r="A87" s="46">
         <v>46104.0</v>
       </c>
@@ -11576,7 +11581,7 @@
       <c r="Z87" s="48"/>
       <c r="AA87" s="48"/>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
+    <row r="88" ht="15.75" hidden="1" customHeight="1">
       <c r="A88" s="46">
         <v>46104.0</v>
       </c>
@@ -11618,7 +11623,7 @@
       <c r="Z88" s="48"/>
       <c r="AA88" s="48"/>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
+    <row r="89" ht="15.75" hidden="1" customHeight="1">
       <c r="A89" s="46">
         <v>46108.0</v>
       </c>
@@ -11660,7 +11665,7 @@
       <c r="Z89" s="48"/>
       <c r="AA89" s="48"/>
     </row>
-    <row r="90" ht="15.75" customHeight="1">
+    <row r="90" ht="15.75" hidden="1" customHeight="1">
       <c r="A90" s="46">
         <v>46108.0</v>
       </c>
@@ -11702,7 +11707,7 @@
       <c r="Z90" s="48"/>
       <c r="AA90" s="48"/>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
+    <row r="91" ht="15.75" hidden="1" customHeight="1">
       <c r="A91" s="46">
         <v>46108.0</v>
       </c>
@@ -11744,7 +11749,7 @@
       <c r="Z91" s="48"/>
       <c r="AA91" s="48"/>
     </row>
-    <row r="92" ht="15.75" customHeight="1">
+    <row r="92" ht="15.75" hidden="1" customHeight="1">
       <c r="A92" s="46">
         <v>46108.0</v>
       </c>
@@ -11786,7 +11791,7 @@
       <c r="Z92" s="48"/>
       <c r="AA92" s="48"/>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
+    <row r="93" ht="15.75" hidden="1" customHeight="1">
       <c r="A93" s="46">
         <v>46108.0</v>
       </c>
@@ -11828,7 +11833,7 @@
       <c r="Z93" s="48"/>
       <c r="AA93" s="48"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
+    <row r="94" ht="15.75" hidden="1" customHeight="1">
       <c r="A94" s="46">
         <v>46108.0</v>
       </c>
@@ -11870,7 +11875,7 @@
       <c r="Z94" s="48"/>
       <c r="AA94" s="48"/>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
+    <row r="95" ht="15.75" hidden="1" customHeight="1">
       <c r="A95" s="46">
         <v>46108.0</v>
       </c>
@@ -11912,7 +11917,7 @@
       <c r="Z95" s="48"/>
       <c r="AA95" s="48"/>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
+    <row r="96" ht="15.75" hidden="1" customHeight="1">
       <c r="A96" s="46">
         <v>46108.0</v>
       </c>
@@ -11954,7 +11959,7 @@
       <c r="Z96" s="48"/>
       <c r="AA96" s="48"/>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
+    <row r="97" ht="15.75" hidden="1" customHeight="1">
       <c r="A97" s="46">
         <v>46108.0</v>
       </c>
@@ -11996,7 +12001,7 @@
       <c r="Z97" s="48"/>
       <c r="AA97" s="48"/>
     </row>
-    <row r="98" ht="15.75" customHeight="1">
+    <row r="98" ht="15.75" hidden="1" customHeight="1">
       <c r="A98" s="46">
         <v>46109.0</v>
       </c>
@@ -12038,7 +12043,7 @@
       <c r="Z98" s="48"/>
       <c r="AA98" s="48"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
+    <row r="99" ht="15.75" hidden="1" customHeight="1">
       <c r="A99" s="46">
         <v>46109.0</v>
       </c>
@@ -12080,7 +12085,7 @@
       <c r="Z99" s="48"/>
       <c r="AA99" s="48"/>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
+    <row r="100" ht="15.75" hidden="1" customHeight="1">
       <c r="A100" s="46">
         <v>46109.0</v>
       </c>
@@ -12122,7 +12127,7 @@
       <c r="Z100" s="48"/>
       <c r="AA100" s="48"/>
     </row>
-    <row r="101" ht="15.75" customHeight="1">
+    <row r="101" ht="15.75" hidden="1" customHeight="1">
       <c r="A101" s="46">
         <v>46109.0</v>
       </c>
@@ -12164,7 +12169,7 @@
       <c r="Z101" s="48"/>
       <c r="AA101" s="48"/>
     </row>
-    <row r="102" ht="15.75" customHeight="1">
+    <row r="102" ht="15.75" hidden="1" customHeight="1">
       <c r="A102" s="46">
         <v>46109.0</v>
       </c>
@@ -12206,7 +12211,7 @@
       <c r="Z102" s="48"/>
       <c r="AA102" s="48"/>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
+    <row r="103" ht="15.75" hidden="1" customHeight="1">
       <c r="A103" s="46">
         <v>46109.0</v>
       </c>
@@ -12248,7 +12253,7 @@
       <c r="Z103" s="48"/>
       <c r="AA103" s="48"/>
     </row>
-    <row r="104" ht="15.75" customHeight="1">
+    <row r="104" ht="15.75" hidden="1" customHeight="1">
       <c r="A104" s="46">
         <v>46109.0</v>
       </c>
@@ -12290,7 +12295,7 @@
       <c r="Z104" s="48"/>
       <c r="AA104" s="48"/>
     </row>
-    <row r="105" ht="15.75" customHeight="1">
+    <row r="105" ht="15.75" hidden="1" customHeight="1">
       <c r="A105" s="46">
         <v>46109.0</v>
       </c>
@@ -12332,7 +12337,7 @@
       <c r="Z105" s="48"/>
       <c r="AA105" s="48"/>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
+    <row r="106" ht="15.75" hidden="1" customHeight="1">
       <c r="A106" s="46">
         <v>46109.0</v>
       </c>
@@ -12374,7 +12379,7 @@
       <c r="Z106" s="48"/>
       <c r="AA106" s="48"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
+    <row r="107" ht="15.75" hidden="1" customHeight="1">
       <c r="A107" s="46">
         <v>46109.0</v>
       </c>
@@ -12416,7 +12421,7 @@
       <c r="Z107" s="48"/>
       <c r="AA107" s="48"/>
     </row>
-    <row r="108" ht="15.75" customHeight="1">
+    <row r="108" ht="15.75" hidden="1" customHeight="1">
       <c r="A108" s="46">
         <v>46109.0</v>
       </c>
@@ -12458,7 +12463,7 @@
       <c r="Z108" s="48"/>
       <c r="AA108" s="48"/>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
+    <row r="109" ht="15.75" hidden="1" customHeight="1">
       <c r="A109" s="46">
         <v>46109.0</v>
       </c>
@@ -12500,7 +12505,7 @@
       <c r="Z109" s="48"/>
       <c r="AA109" s="48"/>
     </row>
-    <row r="110" ht="15.75" customHeight="1">
+    <row r="110" ht="15.75" hidden="1" customHeight="1">
       <c r="A110" s="46">
         <v>46109.0</v>
       </c>
@@ -12542,7 +12547,7 @@
       <c r="Z110" s="48"/>
       <c r="AA110" s="48"/>
     </row>
-    <row r="111" ht="15.75" customHeight="1">
+    <row r="111" ht="15.75" hidden="1" customHeight="1">
       <c r="A111" s="46">
         <v>46109.0</v>
       </c>
@@ -12584,7 +12589,7 @@
       <c r="Z111" s="48"/>
       <c r="AA111" s="48"/>
     </row>
-    <row r="112" ht="15.75" customHeight="1">
+    <row r="112" ht="15.75" hidden="1" customHeight="1">
       <c r="A112" s="46">
         <v>46109.0</v>
       </c>
@@ -12626,7 +12631,7 @@
       <c r="Z112" s="48"/>
       <c r="AA112" s="48"/>
     </row>
-    <row r="113" ht="15.75" customHeight="1">
+    <row r="113" ht="15.75" hidden="1" customHeight="1">
       <c r="A113" s="46">
         <v>46109.0</v>
       </c>
@@ -12668,7 +12673,7 @@
       <c r="Z113" s="48"/>
       <c r="AA113" s="48"/>
     </row>
-    <row r="114" ht="15.75" customHeight="1">
+    <row r="114" ht="15.75" hidden="1" customHeight="1">
       <c r="A114" s="46">
         <v>46109.0</v>
       </c>
@@ -12710,7 +12715,7 @@
       <c r="Z114" s="48"/>
       <c r="AA114" s="48"/>
     </row>
-    <row r="115" ht="15.75" customHeight="1">
+    <row r="115" ht="15.75" hidden="1" customHeight="1">
       <c r="A115" s="46">
         <v>46109.0</v>
       </c>
@@ -12752,7 +12757,7 @@
       <c r="Z115" s="48"/>
       <c r="AA115" s="48"/>
     </row>
-    <row r="116" ht="15.75" customHeight="1">
+    <row r="116" ht="15.75" hidden="1" customHeight="1">
       <c r="A116" s="46">
         <v>46109.0</v>
       </c>
@@ -12794,7 +12799,7 @@
       <c r="Z116" s="48"/>
       <c r="AA116" s="48"/>
     </row>
-    <row r="117" ht="15.75" customHeight="1">
+    <row r="117" ht="15.75" hidden="1" customHeight="1">
       <c r="A117" s="46">
         <v>46109.0</v>
       </c>
@@ -12836,7 +12841,7 @@
       <c r="Z117" s="48"/>
       <c r="AA117" s="48"/>
     </row>
-    <row r="118" ht="15.75" customHeight="1">
+    <row r="118" ht="15.75" hidden="1" customHeight="1">
       <c r="A118" s="46">
         <v>46109.0</v>
       </c>
@@ -12878,7 +12883,7 @@
       <c r="Z118" s="48"/>
       <c r="AA118" s="48"/>
     </row>
-    <row r="119" ht="15.75" customHeight="1">
+    <row r="119" ht="15.75" hidden="1" customHeight="1">
       <c r="A119" s="46">
         <v>46109.0</v>
       </c>
@@ -12920,7 +12925,7 @@
       <c r="Z119" s="48"/>
       <c r="AA119" s="48"/>
     </row>
-    <row r="120" ht="15.75" customHeight="1">
+    <row r="120" ht="15.75" hidden="1" customHeight="1">
       <c r="A120" s="46">
         <v>46109.0</v>
       </c>
@@ -12962,7 +12967,7 @@
       <c r="Z120" s="48"/>
       <c r="AA120" s="48"/>
     </row>
-    <row r="121" ht="15.75" customHeight="1">
+    <row r="121" ht="15.75" hidden="1" customHeight="1">
       <c r="A121" s="46">
         <v>46109.0</v>
       </c>
@@ -13004,7 +13009,7 @@
       <c r="Z121" s="48"/>
       <c r="AA121" s="48"/>
     </row>
-    <row r="122" ht="15.75" customHeight="1">
+    <row r="122" ht="15.75" hidden="1" customHeight="1">
       <c r="A122" s="46">
         <v>46109.0</v>
       </c>
@@ -13046,7 +13051,7 @@
       <c r="Z122" s="48"/>
       <c r="AA122" s="48"/>
     </row>
-    <row r="123" ht="15.75" customHeight="1">
+    <row r="123" ht="15.75" hidden="1" customHeight="1">
       <c r="A123" s="46">
         <v>46109.0</v>
       </c>
@@ -13088,7 +13093,7 @@
       <c r="Z123" s="48"/>
       <c r="AA123" s="48"/>
     </row>
-    <row r="124" ht="15.75" customHeight="1">
+    <row r="124" ht="15.75" hidden="1" customHeight="1">
       <c r="A124" s="46">
         <v>46109.0</v>
       </c>
@@ -13134,9 +13139,7 @@
       <c r="A125" s="46">
         <v>46111.0</v>
       </c>
-      <c r="B125" s="46">
-        <v>46111.0</v>
-      </c>
+      <c r="B125" s="46"/>
       <c r="C125" s="23" t="s">
         <v>83</v>
       </c>
@@ -13176,9 +13179,7 @@
       <c r="A126" s="46">
         <v>46111.0</v>
       </c>
-      <c r="B126" s="46">
-        <v>46111.0</v>
-      </c>
+      <c r="B126" s="46"/>
       <c r="C126" s="23" t="s">
         <v>115</v>
       </c>
@@ -13218,9 +13219,7 @@
       <c r="A127" s="46">
         <v>46111.0</v>
       </c>
-      <c r="B127" s="46">
-        <v>46111.0</v>
-      </c>
+      <c r="B127" s="46"/>
       <c r="C127" s="23" t="s">
         <v>118</v>
       </c>
@@ -13260,9 +13259,7 @@
       <c r="A128" s="46">
         <v>46111.0</v>
       </c>
-      <c r="B128" s="46">
-        <v>46111.0</v>
-      </c>
+      <c r="B128" s="46"/>
       <c r="C128" s="23" t="s">
         <v>126</v>
       </c>
@@ -13302,9 +13299,7 @@
       <c r="A129" s="46">
         <v>46111.0</v>
       </c>
-      <c r="B129" s="46">
-        <v>46111.0</v>
-      </c>
+      <c r="B129" s="46"/>
       <c r="C129" s="23" t="s">
         <v>133</v>
       </c>
@@ -39493,6 +39488,13 @@
       <c r="AA1028" s="48"/>
     </row>
   </sheetData>
+  <autoFilter ref="$A$3:$H$1028">
+    <filterColumn colId="4">
+      <filters blank="1">
+        <filter val="IN-TRANSIT"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>

</xml_diff>